<commit_message>
feat: connect local workspace runtime and secure imports
</commit_message>
<xml_diff>
--- a/templates/import/asset-metadata.xlsx
+++ b/templates/import/asset-metadata.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="1" r:id="R5f5203a949d74e65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导入数据" sheetId="2" r:id="R01211e51e68d4b59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="1" r:id="R4db44ce830594617"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导入数据" sheetId="2" r:id="Rbd53ecca701449a3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,6 +14,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="0"/>
+  </x:numFmts>
   <x:fonts count="2">
     <x:font>
       <x:sz val="11"/>
@@ -26,7 +29,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -48,6 +51,11 @@
         <x:fgColor rgb="FFFFF8DD"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF276BDE"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="10">
     <x:border/>
@@ -145,7 +153,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="28">
+  <x:cellXfs count="33">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -188,6 +196,11 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -567,6 +580,64 @@
       </x:c>
       <x:c r="I6" s="12" t="str"/>
     </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>产品名称</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>productName</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>按现有产品名称匹配</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>演示产品 A</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>文本</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>不适用</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>可为空</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>productName</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>渠道</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>channel</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>抖音/天猫/京东</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>抖音</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>枚举</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>待确认</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>可为空</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>channel</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -576,11 +647,13 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="21" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="21" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="21" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="21" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="21" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="21" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="21" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -599,22 +672,32 @@
       <x:c r="E1" s="18" t="str">
         <x:v>素材来源 (sourceType)</x:v>
       </x:c>
+      <x:c r="F1" s="31" t="str">
+        <x:v>产品名称 (productName)</x:v>
+      </x:c>
+      <x:c r="G1" s="32" t="str">
+        <x:v>渠道 (channel)</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="19" t="str">
-        <x:v>SF-DEMO-001</x:v>
+        <x:v>SF-IMPORT-001</x:v>
       </x:c>
       <x:c r="B2" s="20" t="str">
-        <x:v>匿名素材 01</x:v>
-      </x:c>
-      <x:c r="C2" s="20" t="str">
-        <x:v>待补充</x:v>
-      </x:c>
-      <x:c r="D2" s="20" t="str">
+        <x:v>匿名导入素材 001</x:v>
+      </x:c>
+      <x:c r="C2" s="20"/>
+      <x:c r="D2" s="28" t="n">
         <x:v>18</x:v>
       </x:c>
       <x:c r="E2" s="21" t="str">
         <x:v>原创</x:v>
+      </x:c>
+      <x:c r="F2" s="22" t="str">
+        <x:v>演示产品 A</x:v>
+      </x:c>
+      <x:c r="G2" s="24" t="str">
+        <x:v>抖音</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -623,6 +706,8 @@
       <x:c r="C3" s="23"/>
       <x:c r="D3" s="23"/>
       <x:c r="E3" s="24"/>
+      <x:c r="F3" s="22"/>
+      <x:c r="G3" s="24"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="22"/>
@@ -630,6 +715,8 @@
       <x:c r="C4" s="23"/>
       <x:c r="D4" s="23"/>
       <x:c r="E4" s="24"/>
+      <x:c r="F4" s="22"/>
+      <x:c r="G4" s="24"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="22"/>
@@ -637,6 +724,8 @@
       <x:c r="C5" s="23"/>
       <x:c r="D5" s="23"/>
       <x:c r="E5" s="24"/>
+      <x:c r="F5" s="22"/>
+      <x:c r="G5" s="24"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="22"/>
@@ -644,6 +733,8 @@
       <x:c r="C6" s="23"/>
       <x:c r="D6" s="23"/>
       <x:c r="E6" s="24"/>
+      <x:c r="F6" s="22"/>
+      <x:c r="G6" s="24"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="22"/>
@@ -651,6 +742,8 @@
       <x:c r="C7" s="23"/>
       <x:c r="D7" s="23"/>
       <x:c r="E7" s="24"/>
+      <x:c r="F7" s="22"/>
+      <x:c r="G7" s="24"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="22"/>
@@ -658,6 +751,8 @@
       <x:c r="C8" s="23"/>
       <x:c r="D8" s="23"/>
       <x:c r="E8" s="24"/>
+      <x:c r="F8" s="22"/>
+      <x:c r="G8" s="24"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="22"/>
@@ -665,6 +760,8 @@
       <x:c r="C9" s="23"/>
       <x:c r="D9" s="23"/>
       <x:c r="E9" s="24"/>
+      <x:c r="F9" s="22"/>
+      <x:c r="G9" s="24"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="22"/>
@@ -672,6 +769,8 @@
       <x:c r="C10" s="23"/>
       <x:c r="D10" s="23"/>
       <x:c r="E10" s="24"/>
+      <x:c r="F10" s="22"/>
+      <x:c r="G10" s="24"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="22"/>
@@ -679,6 +778,8 @@
       <x:c r="C11" s="23"/>
       <x:c r="D11" s="23"/>
       <x:c r="E11" s="24"/>
+      <x:c r="F11" s="22"/>
+      <x:c r="G11" s="24"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="22"/>
@@ -686,6 +787,8 @@
       <x:c r="C12" s="23"/>
       <x:c r="D12" s="23"/>
       <x:c r="E12" s="24"/>
+      <x:c r="F12" s="22"/>
+      <x:c r="G12" s="24"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="22"/>
@@ -693,6 +796,8 @@
       <x:c r="C13" s="23"/>
       <x:c r="D13" s="23"/>
       <x:c r="E13" s="24"/>
+      <x:c r="F13" s="22"/>
+      <x:c r="G13" s="24"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="22"/>
@@ -700,6 +805,8 @@
       <x:c r="C14" s="23"/>
       <x:c r="D14" s="23"/>
       <x:c r="E14" s="24"/>
+      <x:c r="F14" s="22"/>
+      <x:c r="G14" s="24"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="22"/>
@@ -707,6 +814,8 @@
       <x:c r="C15" s="23"/>
       <x:c r="D15" s="23"/>
       <x:c r="E15" s="24"/>
+      <x:c r="F15" s="22"/>
+      <x:c r="G15" s="24"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="22"/>
@@ -714,6 +823,8 @@
       <x:c r="C16" s="23"/>
       <x:c r="D16" s="23"/>
       <x:c r="E16" s="24"/>
+      <x:c r="F16" s="22"/>
+      <x:c r="G16" s="24"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="22"/>
@@ -721,6 +832,8 @@
       <x:c r="C17" s="23"/>
       <x:c r="D17" s="23"/>
       <x:c r="E17" s="24"/>
+      <x:c r="F17" s="22"/>
+      <x:c r="G17" s="24"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="22"/>
@@ -728,6 +841,8 @@
       <x:c r="C18" s="23"/>
       <x:c r="D18" s="23"/>
       <x:c r="E18" s="24"/>
+      <x:c r="F18" s="22"/>
+      <x:c r="G18" s="24"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="22"/>
@@ -735,6 +850,8 @@
       <x:c r="C19" s="23"/>
       <x:c r="D19" s="23"/>
       <x:c r="E19" s="24"/>
+      <x:c r="F19" s="22"/>
+      <x:c r="G19" s="24"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="25"/>
@@ -742,6 +859,8 @@
       <x:c r="C20" s="26"/>
       <x:c r="D20" s="26"/>
       <x:c r="E20" s="27"/>
+      <x:c r="F20" s="25"/>
+      <x:c r="G20" s="27"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
docs: prepare bilingual public release
</commit_message>
<xml_diff>
--- a/templates/import/asset-metadata.xlsx
+++ b/templates/import/asset-metadata.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="1" r:id="R4db44ce830594617"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导入数据" sheetId="2" r:id="Rbd53ecca701449a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="1" r:id="R8df3ad82262043bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导入数据" sheetId="2" r:id="Rf8d4cd4f7214496e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -617,10 +617,10 @@
         <x:v>channel</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>抖音/天猫/京东</x:v>
+        <x:v>Built-in or custom platform name / 内置或自定义平台名称</x:v>
       </x:c>
       <x:c r="D8" t="str">
-        <x:v>抖音</x:v>
+        <x:v>TikTok Shop</x:v>
       </x:c>
       <x:c r="E8" t="str">
         <x:v>否</x:v>
@@ -697,7 +697,7 @@
         <x:v>演示产品 A</x:v>
       </x:c>
       <x:c r="G2" s="24" t="str">
-        <x:v>抖音</x:v>
+        <x:v>TikTok Shop</x:v>
       </x:c>
     </x:row>
     <x:row r="3">

</xml_diff>